<commit_message>
B4 and B6: final corrections on the 24 September runs
B4 re-priced on the revised framework's blended conversion rate (group
rate standing in for the child's) and a corrected group CVR roll-up.
B6 re-validated on run 20260924-981b2555 (focus Queen, Full, King,
Cooling): push inside the loss stop, engine-plan envelope and TACoS
guard; out-of-focus test with the flagship held; freezes on the 7-day
median; rows that should not load; Part D rebuilt for B6.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvXHKtbYmE3ru99HYV2muV
</commit_message>
<xml_diff>
--- a/docs/DBS4_Corrections_by_Situation_20260924-5e8a0f10.xlsx
+++ b/docs/DBS4_Corrections_by_Situation_20260924-5e8a0f10.xlsx
@@ -665,7 +665,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Push TOS +30% (12% of required top-of-search clicks delivered → +30%): $5.71 → $7.43; modifier 446%; investigate the rank loss the same day; re-point the ad to the serving child; daily read to 09-28</t>
+          <t>Push TOS +30% (12% of required top-of-search clicks delivered → +30%; stopped at the loss stop 7.31): $5.71 → $7.31; modifier 437%; investigate the rank loss the same day; re-point the ad to the serving child; daily read to 09-28</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Push TOS +0% (loss stop — no top-of-search order on its 15 top-of-search clicks in 90 days: no step until it converts): $4.80 → $4.80; modifier 253%; re-point the ad to the serving child; daily read to 09-28</t>
+          <t>Push TOS +30% (10% of required top-of-search clicks delivered → +30%): $4.80 → $6.24; modifier 359%; re-point the ad to the serving child; daily read to 09-28</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Push TOS +30% (20% of required top-of-search clicks delivered → +30%; stopped at the loss stop 12.96): $10.35 → $12.96; modifier 319%; re-point the ad to the serving child; daily read to 09-28</t>
+          <t>Push TOS +0% (loss stop reached — at 10.35 a top-of-search order already costs 123 (stop 3× contribution = 87)): $10.35 → $10.35; modifier 235%; re-point the ad to the serving child; daily read to 09-28</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Push TOS +30% (3% of required top-of-search clicks delivered → +30%): $5.80 → $7.55; modifier 180%; re-point the ad to the serving child; daily read to 09-28</t>
+          <t>Push TOS +30% (3% of required top-of-search clicks delivered → +30%; stopped at the loss stop 6.73): $5.80 → $6.73; modifier 149%; re-point the ad to the serving child; daily read to 09-28</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Push TOS +20% (no click requirement on file → +20% (a stated departure: the logic document would hold at the ceiling); stopped at the loss stop 12.12): $10.41 → $12.12; modifier 304%; daily read to 09-28</t>
+          <t>Push TOS +20% (no click requirement on file → +20% (a stated departure: the logic document would hold at the ceiling); stopped at the loss stop 11.53): $10.41 → $11.53; modifier 284%; daily read to 09-28</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Out of focus but converts (25% at top of search vs bar 10.8%): test TOS +10% $4.87 → $5.35 to 10-08; budget $5.74/day</t>
+          <t>Out of focus but converts (14% at top of search vs bar 10.8%): test TOS +10% $4.87 → $5.35 to 10-08; budget $5.74/day</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Out of focus but converts (31% at top of search vs bar 10.5%): test TOS +10% $4.95 → $5.45 to 10-08; budget $8.00/day</t>
+          <t>Out of focus but converts (18% at top of search vs bar 10.5%): test TOS +10% $4.95 → $5.45 to 10-08; budget $8.00/day</t>
         </is>
       </c>
     </row>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Out of focus but converts (20% at top of search vs bar 18.6%): test TOS +10% $2.41 → $2.65 to 10-08; budget $5.00/day</t>
+          <t>Out of focus but converts (14% at top of search vs bar 18.6%): test TOS +10% $2.41 → $2.65 to 10-08; budget $5.00/day</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2736,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Out of focus but converts (18% at top of search vs bar 11.5%): test TOS +10% $6.40 → $7.04 to 10-08; budget $12.00/day</t>
+          <t>Out of focus but converts (16% at top of search vs bar 11.5%): test TOS +10% $6.40 → $7.04 to 10-08; budget $12.00/day</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Out of focus but converts (29% at top of search vs bar 16.5%): test TOS +10% $8.74 → $9.61 to 10-08; budget $10.30/day</t>
+          <t>Out of focus but converts (23% at top of search vs bar 16.5%): test TOS +10% $8.74 → $9.61 to 10-08; budget $10.30/day</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Out of focus but converts (8% at top of search vs bar 7.4%): test TOS +10% $2.66 → $2.93 to 10-08; budget $26.00/day</t>
+          <t>Out of focus but converts (9% at top of search vs bar 7.4%): test TOS +10% $2.66 → $2.93 to 10-08; budget $26.00/day</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>Out of focus but converts (30% at top of search vs bar 13.3%): test TOS +10% $4.71 → $5.18 to 10-08; budget $30.00/day</t>
+          <t>Out of focus but converts (20% at top of search vs bar 13.3%): test TOS +10% $4.71 → $5.18 to 10-08; budget $30.00/day</t>
         </is>
       </c>
     </row>
@@ -20132,7 +20132,7 @@
         <v>1.91</v>
       </c>
       <c r="I2" t="n">
-        <v>13.73</v>
+        <v>13.93</v>
       </c>
       <c r="J2" t="n">
         <v>8.279999999999999</v>
@@ -20191,7 +20191,7 @@
         <v>2.1</v>
       </c>
       <c r="I3" t="n">
-        <v>8.49</v>
+        <v>8.77</v>
       </c>
       <c r="J3" t="n">
         <v>8.699999999999999</v>
@@ -20213,7 +20213,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>PERFORMANCE GAP — shown, but CVR under target</t>
+          <t>MEETS THE BARS — impression share not read</t>
         </is>
       </c>
     </row>
@@ -20247,7 +20247,7 @@
         <v>1.94</v>
       </c>
       <c r="I4" t="n">
-        <v>14.9</v>
+        <v>18.76</v>
       </c>
       <c r="J4" t="n">
         <v>10.83</v>
@@ -20306,7 +20306,7 @@
         <v>1.79</v>
       </c>
       <c r="I5" t="n">
-        <v>21.91</v>
+        <v>23.72</v>
       </c>
       <c r="J5" t="n">
         <v>13.26</v>
@@ -20365,7 +20365,7 @@
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>14.47</v>
+        <v>19.7</v>
       </c>
       <c r="J6" t="n">
         <v>13.2</v>
@@ -20375,7 +20375,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON TRACK</t>
+          <t>MEETS THE BARS — impression share not read</t>
         </is>
       </c>
     </row>
@@ -20409,7 +20409,7 @@
         <v>2.18</v>
       </c>
       <c r="I7" t="n">
-        <v>22.65</v>
+        <v>23.8</v>
       </c>
       <c r="J7" t="n">
         <v>12.09</v>
@@ -20468,7 +20468,7 @@
         <v>2.07</v>
       </c>
       <c r="I8" t="n">
-        <v>19.09</v>
+        <v>21.41</v>
       </c>
       <c r="J8" t="n">
         <v>7.5</v>
@@ -20527,7 +20527,7 @@
         <v>2.15</v>
       </c>
       <c r="I9" t="n">
-        <v>17.87</v>
+        <v>30.78</v>
       </c>
       <c r="J9" t="n">
         <v>10.5</v>
@@ -20586,7 +20586,7 @@
         <v>2.06</v>
       </c>
       <c r="I10" t="n">
-        <v>25.33</v>
+        <v>31.03</v>
       </c>
       <c r="J10" t="n">
         <v>12.18</v>
@@ -20645,7 +20645,7 @@
         <v>1.85</v>
       </c>
       <c r="I11" t="n">
-        <v>19.16</v>
+        <v>21.57</v>
       </c>
       <c r="J11" t="n">
         <v>17.1</v>
@@ -20655,7 +20655,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>ON TRACK</t>
+          <t>MEETS THE BARS — impression share not read</t>
         </is>
       </c>
     </row>
@@ -20689,7 +20689,7 @@
         <v>1.81</v>
       </c>
       <c r="I12" t="n">
-        <v>19.92</v>
+        <v>24.92</v>
       </c>
       <c r="J12" t="n">
         <v>18.3</v>
@@ -20699,7 +20699,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ON TRACK</t>
+          <t>MEETS THE BARS — impression share not read</t>
         </is>
       </c>
     </row>
@@ -20733,7 +20733,7 @@
         <v>2.07</v>
       </c>
       <c r="I13" t="n">
-        <v>30.43</v>
+        <v>34.4</v>
       </c>
       <c r="J13" t="n">
         <v>10.98</v>
@@ -20792,7 +20792,7 @@
         <v>2.07</v>
       </c>
       <c r="I14" t="n">
-        <v>10.06</v>
+        <v>25.62</v>
       </c>
       <c r="J14" t="n">
         <v>8.82</v>
@@ -20851,7 +20851,7 @@
         <v>1.94</v>
       </c>
       <c r="I15" t="n">
-        <v>6.27</v>
+        <v>18.23</v>
       </c>
       <c r="J15" t="n">
         <v>16.02</v>
@@ -20861,7 +20861,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>BOTH — short of traffic and under target</t>
+          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
         </is>
       </c>
     </row>
@@ -20895,7 +20895,7 @@
         <v>1.8</v>
       </c>
       <c r="I16" t="n">
-        <v>26.87</v>
+        <v>31.21</v>
       </c>
       <c r="J16" t="n">
         <v>21.21</v>
@@ -20905,7 +20905,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>ON TRACK</t>
+          <t>MEETS THE BARS — impression share not read</t>
         </is>
       </c>
     </row>
@@ -20939,7 +20939,7 @@
         <v>2.17</v>
       </c>
       <c r="I17" t="n">
-        <v>15.69</v>
+        <v>24.12</v>
       </c>
       <c r="J17" t="n">
         <v>12.51</v>
@@ -21050,14 +21050,8 @@
       <c r="F19" t="n">
         <v>91</v>
       </c>
-      <c r="G19" t="n">
-        <v>18.41</v>
-      </c>
       <c r="H19" t="n">
         <v>2.1</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0</v>
       </c>
       <c r="J19" t="n">
         <v>10.05</v>

</xml_diff>